<commit_message>
add 3D earth project NODEJS
</commit_message>
<xml_diff>
--- a/气象/蒙古存档.xlsx
+++ b/气象/蒙古存档.xlsx
@@ -18411,45 +18411,45 @@
       <c r="A394" s="1" t="n">
         <v>46153</v>
       </c>
-      <c r="B394" t="n">
+      <c r="B394" s="0" t="n">
         <v>9.699999999999999</v>
       </c>
-      <c r="C394" t="n">
+      <c r="C394" s="0" t="n">
         <v>9.699999999999999</v>
       </c>
-      <c r="D394" t="n">
+      <c r="D394" s="0" t="n">
         <v>12.6</v>
       </c>
-      <c r="E394" t="inlineStr">
-        <is>
-          <t>无</t>
-        </is>
-      </c>
-      <c r="F394" t="n">
+      <c r="E394" s="0" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="F394" s="0" t="n">
         <v>5.4</v>
       </c>
-      <c r="G394" t="n">
+      <c r="G394" s="0" t="n">
         <v>7.1</v>
       </c>
-      <c r="H394" t="n">
+      <c r="H394" s="0" t="n">
         <v>8.699999999999999</v>
       </c>
-      <c r="I394" t="n">
+      <c r="I394" s="0" t="n">
         <v>8.9</v>
       </c>
-      <c r="J394" t="n">
+      <c r="J394" s="0" t="n">
         <v>11.2</v>
       </c>
-      <c r="K394" t="n">
+      <c r="K394" s="0" t="n">
         <v>7.6</v>
       </c>
-      <c r="L394" t="n">
+      <c r="L394" s="0" t="n">
         <v>7.4</v>
       </c>
-      <c r="M394" t="n">
+      <c r="M394" s="0" t="n">
         <v>7.6</v>
       </c>
-      <c r="N394" t="n">
+      <c r="N394" s="0" t="n">
         <v>12.8</v>
       </c>
     </row>
@@ -18457,35 +18457,324 @@
       <c r="A395" s="1" t="n">
         <v>46154</v>
       </c>
+      <c r="B395" s="0" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="C395" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="D395" s="0" t="n">
+        <v>7.4</v>
+      </c>
+      <c r="E395" s="0" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="F395" s="0" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="G395" s="0" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="H395" s="0" t="n">
+        <v>8.1</v>
+      </c>
+      <c r="I395" s="0" t="n">
+        <v>5.8</v>
+      </c>
+      <c r="J395" s="0" t="n">
+        <v>5.4</v>
+      </c>
+      <c r="K395" s="0" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="L395" s="0" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="M395" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="N395" s="0" t="n">
+        <v>12.4</v>
+      </c>
     </row>
     <row r="396">
       <c r="A396" s="1" t="n">
         <v>46155</v>
       </c>
+      <c r="B396" s="0" t="n">
+        <v>-3.6</v>
+      </c>
+      <c r="C396" s="0" t="n">
+        <v>-0.8</v>
+      </c>
+      <c r="D396" s="0" t="n">
+        <v>-3.1</v>
+      </c>
+      <c r="E396" s="0" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="F396" s="0" t="n">
+        <v>-0.2</v>
+      </c>
+      <c r="G396" s="0" t="n">
+        <v>-2.9</v>
+      </c>
+      <c r="H396" s="0" t="n">
+        <v>5.4</v>
+      </c>
+      <c r="I396" s="0" t="n">
+        <v>-0.7</v>
+      </c>
+      <c r="J396" s="0" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="K396" s="0" t="n">
+        <v>-5.6</v>
+      </c>
+      <c r="L396" s="0" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="M396" s="0" t="n">
+        <v>-3.6</v>
+      </c>
+      <c r="N396" s="0" t="n">
+        <v>6.1</v>
+      </c>
     </row>
     <row r="397">
       <c r="A397" s="1" t="n">
         <v>46156</v>
       </c>
+      <c r="B397" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="C397" s="0" t="n">
+        <v>-1.7</v>
+      </c>
+      <c r="D397" s="0" t="n">
+        <v>-4.5</v>
+      </c>
+      <c r="E397" s="0" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="F397" s="0" t="n">
+        <v>-8.9</v>
+      </c>
+      <c r="G397" s="0" t="n">
+        <v>-8.1</v>
+      </c>
+      <c r="H397" s="0" t="n">
+        <v>-3.4</v>
+      </c>
+      <c r="I397" s="0" t="n">
+        <v>-1.3</v>
+      </c>
+      <c r="J397" s="0" t="n">
+        <v>-6.1</v>
+      </c>
+      <c r="K397" s="0" t="n">
+        <v>-5.8</v>
+      </c>
+      <c r="L397" s="0" t="n">
+        <v>-6</v>
+      </c>
+      <c r="M397" s="0" t="n">
+        <v>-8.9</v>
+      </c>
+      <c r="N397" s="0" t="n">
+        <v>3.8</v>
+      </c>
     </row>
     <row r="398">
       <c r="A398" s="1" t="n">
         <v>46157</v>
       </c>
+      <c r="B398" s="0" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="C398" s="0" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="D398" s="0" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="E398" s="0" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="F398" s="0" t="n">
+        <v>-2.6</v>
+      </c>
+      <c r="G398" s="0" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="H398" s="0" t="n">
+        <v>-1.3</v>
+      </c>
+      <c r="I398" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="J398" s="0" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="K398" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="L398" s="0" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="M398" s="0" t="n">
+        <v>-0.2</v>
+      </c>
+      <c r="N398" s="0" t="n">
+        <v>1.6</v>
+      </c>
     </row>
     <row r="399">
       <c r="A399" s="1" t="n">
         <v>46158</v>
       </c>
+      <c r="B399" s="0" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="C399" s="0" t="n">
+        <v>-0.2</v>
+      </c>
+      <c r="D399" s="0" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="E399" s="0" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="F399" s="0" t="n">
+        <v>-2.7</v>
+      </c>
+      <c r="G399" s="0" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="H399" s="0" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="I399" s="0" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="J399" s="0" t="n">
+        <v>-0.2</v>
+      </c>
+      <c r="K399" s="0" t="n">
+        <v>-0.7</v>
+      </c>
+      <c r="L399" s="0" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="M399" s="0" t="n">
+        <v>-0.2</v>
+      </c>
+      <c r="N399" s="0" t="n">
+        <v>9.699999999999999</v>
+      </c>
     </row>
     <row r="400">
       <c r="A400" s="1" t="n">
         <v>46159</v>
       </c>
+      <c r="B400" s="0" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="C400" s="0" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="D400" s="0" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="E400" s="0" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="F400" s="0" t="n">
+        <v>-4.1</v>
+      </c>
+      <c r="G400" s="0" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="H400" s="0" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="I400" s="0" t="n">
+        <v>-0.4</v>
+      </c>
+      <c r="J400" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="K400" s="0" t="n">
+        <v>-2.9</v>
+      </c>
+      <c r="L400" s="0" t="n">
+        <v>-0.8</v>
+      </c>
+      <c r="M400" s="0" t="n">
+        <v>-0.1</v>
+      </c>
+      <c r="N400" s="0" t="n">
+        <v>4.9</v>
+      </c>
     </row>
     <row r="401">
       <c r="A401" s="1" t="n">
         <v>46160</v>
+      </c>
+      <c r="B401" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="C401" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="D401" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="E401" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="F401" t="n">
+        <v>-6.3</v>
+      </c>
+      <c r="G401" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="H401" t="n">
+        <v>-0.6</v>
+      </c>
+      <c r="I401" t="n">
+        <v>1</v>
+      </c>
+      <c r="J401" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="K401" t="n">
+        <v>-1.6</v>
+      </c>
+      <c r="L401" t="n">
+        <v>-0.6</v>
+      </c>
+      <c r="M401" t="n">
+        <v>-1</v>
+      </c>
+      <c r="N401" t="n">
+        <v>0.7</v>
       </c>
     </row>
     <row r="402">
@@ -36616,45 +36905,45 @@
       <c r="A394" s="1" t="n">
         <v>46153</v>
       </c>
-      <c r="B394" t="n">
+      <c r="B394" s="0" t="n">
         <v>26.1</v>
       </c>
-      <c r="C394" t="n">
+      <c r="C394" s="0" t="n">
         <v>25.5</v>
       </c>
-      <c r="D394" t="n">
+      <c r="D394" s="0" t="n">
         <v>23.7</v>
       </c>
-      <c r="E394" t="inlineStr">
-        <is>
-          <t>无</t>
-        </is>
-      </c>
-      <c r="F394" t="n">
+      <c r="E394" s="0" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="F394" s="0" t="n">
         <v>21.5</v>
       </c>
-      <c r="G394" t="n">
+      <c r="G394" s="0" t="n">
         <v>17.5</v>
       </c>
-      <c r="H394" t="n">
+      <c r="H394" s="0" t="n">
         <v>27</v>
       </c>
-      <c r="I394" t="n">
+      <c r="I394" s="0" t="n">
         <v>23.1</v>
       </c>
-      <c r="J394" t="n">
+      <c r="J394" s="0" t="n">
         <v>21.6</v>
       </c>
-      <c r="K394" t="n">
+      <c r="K394" s="0" t="n">
         <v>18.1</v>
       </c>
-      <c r="L394" t="n">
+      <c r="L394" s="0" t="n">
         <v>20.7</v>
       </c>
-      <c r="M394" t="n">
+      <c r="M394" s="0" t="n">
         <v>18.9</v>
       </c>
-      <c r="N394" t="n">
+      <c r="N394" s="0" t="n">
         <v>28.1</v>
       </c>
     </row>
@@ -36662,35 +36951,324 @@
       <c r="A395" s="1" t="n">
         <v>46154</v>
       </c>
+      <c r="B395" s="0" t="n">
+        <v>24.8</v>
+      </c>
+      <c r="C395" s="0" t="n">
+        <v>23.3</v>
+      </c>
+      <c r="D395" s="0" t="n">
+        <v>19.2</v>
+      </c>
+      <c r="E395" s="0" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="F395" s="0" t="n">
+        <v>19.3</v>
+      </c>
+      <c r="G395" s="0" t="n">
+        <v>14.5</v>
+      </c>
+      <c r="H395" s="0" t="n">
+        <v>26.5</v>
+      </c>
+      <c r="I395" s="0" t="n">
+        <v>21</v>
+      </c>
+      <c r="J395" s="0" t="n">
+        <v>17.6</v>
+      </c>
+      <c r="K395" s="0" t="n">
+        <v>13.2</v>
+      </c>
+      <c r="L395" s="0" t="n">
+        <v>17.4</v>
+      </c>
+      <c r="M395" s="0" t="n">
+        <v>15</v>
+      </c>
+      <c r="N395" s="0" t="n">
+        <v>30.9</v>
+      </c>
     </row>
     <row r="396">
       <c r="A396" s="1" t="n">
         <v>46155</v>
       </c>
+      <c r="B396" s="0" t="n">
+        <v>14</v>
+      </c>
+      <c r="C396" s="0" t="n">
+        <v>13.7</v>
+      </c>
+      <c r="D396" s="0" t="n">
+        <v>12.9</v>
+      </c>
+      <c r="E396" s="0" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="F396" s="0" t="n">
+        <v>9.800000000000001</v>
+      </c>
+      <c r="G396" s="0" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="H396" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="I396" s="0" t="n">
+        <v>15.4</v>
+      </c>
+      <c r="J396" s="0" t="n">
+        <v>11.2</v>
+      </c>
+      <c r="K396" s="0" t="n">
+        <v>7.1</v>
+      </c>
+      <c r="L396" s="0" t="n">
+        <v>13.9</v>
+      </c>
+      <c r="M396" s="0" t="n">
+        <v>8.6</v>
+      </c>
+      <c r="N396" s="0" t="n">
+        <v>21.2</v>
+      </c>
     </row>
     <row r="397">
       <c r="A397" s="1" t="n">
         <v>46156</v>
       </c>
+      <c r="B397" s="0" t="n">
+        <v>17.3</v>
+      </c>
+      <c r="C397" s="0" t="n">
+        <v>15.4</v>
+      </c>
+      <c r="D397" s="0" t="n">
+        <v>15</v>
+      </c>
+      <c r="E397" s="0" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="F397" s="0" t="n">
+        <v>13.3</v>
+      </c>
+      <c r="G397" s="0" t="n">
+        <v>10.4</v>
+      </c>
+      <c r="H397" s="0" t="n">
+        <v>16.9</v>
+      </c>
+      <c r="I397" s="0" t="n">
+        <v>14.2</v>
+      </c>
+      <c r="J397" s="0" t="n">
+        <v>14</v>
+      </c>
+      <c r="K397" s="0" t="n">
+        <v>11.6</v>
+      </c>
+      <c r="L397" s="0" t="n">
+        <v>15.6</v>
+      </c>
+      <c r="M397" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="N397" s="0" t="n">
+        <v>11.3</v>
+      </c>
     </row>
     <row r="398">
       <c r="A398" s="1" t="n">
         <v>46157</v>
       </c>
+      <c r="B398" s="0" t="n">
+        <v>14.6</v>
+      </c>
+      <c r="C398" s="0" t="n">
+        <v>12.3</v>
+      </c>
+      <c r="D398" s="0" t="n">
+        <v>14.1</v>
+      </c>
+      <c r="E398" s="0" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="F398" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="G398" s="0" t="n">
+        <v>8.6</v>
+      </c>
+      <c r="H398" s="0" t="n">
+        <v>18.5</v>
+      </c>
+      <c r="I398" s="0" t="n">
+        <v>10.4</v>
+      </c>
+      <c r="J398" s="0" t="n">
+        <v>14.3</v>
+      </c>
+      <c r="K398" s="0" t="n">
+        <v>10.2</v>
+      </c>
+      <c r="L398" s="0" t="n">
+        <v>12.8</v>
+      </c>
+      <c r="M398" s="0" t="n">
+        <v>8.800000000000001</v>
+      </c>
+      <c r="N398" s="0" t="n">
+        <v>18.5</v>
+      </c>
     </row>
     <row r="399">
       <c r="A399" s="1" t="n">
         <v>46158</v>
       </c>
+      <c r="B399" s="0" t="n">
+        <v>9.4</v>
+      </c>
+      <c r="C399" s="0" t="n">
+        <v>6.6</v>
+      </c>
+      <c r="D399" s="0" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="E399" s="0" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="F399" s="0" t="n">
+        <v>7.7</v>
+      </c>
+      <c r="G399" s="0" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="H399" s="0" t="n">
+        <v>18.5</v>
+      </c>
+      <c r="I399" s="0" t="n">
+        <v>9.6</v>
+      </c>
+      <c r="J399" s="0" t="n">
+        <v>11.2</v>
+      </c>
+      <c r="K399" s="0" t="n">
+        <v>8</v>
+      </c>
+      <c r="L399" s="0" t="n">
+        <v>11.4</v>
+      </c>
+      <c r="M399" s="0" t="n">
+        <v>6.7</v>
+      </c>
+      <c r="N399" s="0" t="n">
+        <v>17.4</v>
+      </c>
     </row>
     <row r="400">
       <c r="A400" s="1" t="n">
         <v>46159</v>
       </c>
+      <c r="B400" s="0" t="n">
+        <v>15.3</v>
+      </c>
+      <c r="C400" s="0" t="n">
+        <v>13.8</v>
+      </c>
+      <c r="D400" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="E400" s="0" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="F400" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="G400" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="H400" s="0" t="n">
+        <v>16.8</v>
+      </c>
+      <c r="I400" s="0" t="n">
+        <v>17.5</v>
+      </c>
+      <c r="J400" s="0" t="n">
+        <v>5.1</v>
+      </c>
+      <c r="K400" s="0" t="n">
+        <v>5.6</v>
+      </c>
+      <c r="L400" s="0" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="M400" s="0" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="N400" s="0" t="n">
+        <v>15.6</v>
+      </c>
     </row>
     <row r="401">
       <c r="A401" s="1" t="n">
         <v>46160</v>
+      </c>
+      <c r="B401" t="n">
+        <v>12.6</v>
+      </c>
+      <c r="C401" t="n">
+        <v>12</v>
+      </c>
+      <c r="D401" t="n">
+        <v>7.8</v>
+      </c>
+      <c r="E401" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="F401" t="n">
+        <v>9</v>
+      </c>
+      <c r="G401" t="n">
+        <v>7.6</v>
+      </c>
+      <c r="H401" t="n">
+        <v>16.9</v>
+      </c>
+      <c r="I401" t="n">
+        <v>13.3</v>
+      </c>
+      <c r="J401" t="n">
+        <v>9.300000000000001</v>
+      </c>
+      <c r="K401" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="L401" t="n">
+        <v>7.4</v>
+      </c>
+      <c r="M401" t="n">
+        <v>7.4</v>
+      </c>
+      <c r="N401" t="n">
+        <v>15.2</v>
       </c>
     </row>
     <row r="402">
@@ -45087,51 +45665,51 @@
       <c r="A152" s="1" t="n">
         <v>46153</v>
       </c>
-      <c r="B152" t="n">
+      <c r="B152" s="0" t="n">
         <v>19.53</v>
       </c>
-      <c r="C152" t="inlineStr">
-        <is>
-          <t>无</t>
-        </is>
-      </c>
-      <c r="D152" t="inlineStr">
-        <is>
-          <t>无</t>
-        </is>
-      </c>
-      <c r="E152" t="inlineStr">
-        <is>
-          <t>无</t>
-        </is>
-      </c>
-      <c r="F152" t="n">
+      <c r="C152" s="0" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="D152" s="0" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="E152" s="0" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="F152" s="0" t="n">
         <v>15.06</v>
       </c>
-      <c r="G152" t="inlineStr">
-        <is>
-          <t>无</t>
-        </is>
-      </c>
-      <c r="H152" t="n">
+      <c r="G152" s="0" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="H152" s="0" t="n">
         <v>17.49</v>
       </c>
-      <c r="I152" t="n">
+      <c r="I152" s="0" t="n">
         <v>18.73</v>
       </c>
-      <c r="J152" t="n">
+      <c r="J152" s="0" t="n">
         <v>17.05</v>
       </c>
-      <c r="K152" t="n">
+      <c r="K152" s="0" t="n">
         <v>13.2</v>
       </c>
-      <c r="L152" t="n">
+      <c r="L152" s="0" t="n">
         <v>14.04</v>
       </c>
-      <c r="M152" t="n">
+      <c r="M152" s="0" t="n">
         <v>12.53</v>
       </c>
-      <c r="N152" t="n">
+      <c r="N152" s="0" t="n">
         <v>20.34</v>
       </c>
     </row>
@@ -45139,35 +45717,364 @@
       <c r="A153" s="1" t="n">
         <v>46154</v>
       </c>
+      <c r="B153" s="0" t="n">
+        <v>9.91</v>
+      </c>
+      <c r="C153" s="0" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="D153" s="0" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="E153" s="0" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="F153" s="0" t="n">
+        <v>13.14</v>
+      </c>
+      <c r="G153" s="0" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="H153" s="0" t="n">
+        <v>15.95</v>
+      </c>
+      <c r="I153" s="0" t="n">
+        <v>9.42</v>
+      </c>
+      <c r="J153" s="0" t="n">
+        <v>9.33</v>
+      </c>
+      <c r="K153" s="0" t="n">
+        <v>9.130000000000001</v>
+      </c>
+      <c r="L153" s="0" t="n">
+        <v>11.45</v>
+      </c>
+      <c r="M153" s="0" t="n">
+        <v>7.16</v>
+      </c>
+      <c r="N153" s="0" t="n">
+        <v>21.22</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="1" t="n">
         <v>46155</v>
       </c>
+      <c r="B154" s="0" t="n">
+        <v>6.82</v>
+      </c>
+      <c r="C154" s="0" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="D154" s="0" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="E154" s="0" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="F154" s="0" t="n">
+        <v>4.59</v>
+      </c>
+      <c r="G154" s="0" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="H154" s="0" t="n">
+        <v>7.86</v>
+      </c>
+      <c r="I154" s="0" t="n">
+        <v>8.06</v>
+      </c>
+      <c r="J154" s="0" t="n">
+        <v>5.33</v>
+      </c>
+      <c r="K154" s="0" t="n">
+        <v>1.85</v>
+      </c>
+      <c r="L154" s="0" t="n">
+        <v>6.15</v>
+      </c>
+      <c r="M154" s="0" t="n">
+        <v>2.36</v>
+      </c>
+      <c r="N154" s="0" t="n">
+        <v>9.630000000000001</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="1" t="n">
         <v>46156</v>
       </c>
+      <c r="B155" s="0" t="n">
+        <v>9.15</v>
+      </c>
+      <c r="C155" s="0" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="D155" s="0" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="E155" s="0" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="F155" s="0" t="n">
+        <v>2.86</v>
+      </c>
+      <c r="G155" s="0" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="H155" s="0" t="n">
+        <v>7.1</v>
+      </c>
+      <c r="I155" s="0" t="n">
+        <v>6.95</v>
+      </c>
+      <c r="J155" s="0" t="n">
+        <v>5.54</v>
+      </c>
+      <c r="K155" s="0" t="n">
+        <v>3.71</v>
+      </c>
+      <c r="L155" s="0" t="n">
+        <v>5.39</v>
+      </c>
+      <c r="M155" s="0" t="n">
+        <v>2.08</v>
+      </c>
+      <c r="N155" s="0" t="n">
+        <v>7.65</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="1" t="n">
         <v>46157</v>
       </c>
+      <c r="B156" s="0" t="n">
+        <v>8.17</v>
+      </c>
+      <c r="C156" s="0" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="D156" s="0" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="E156" s="0" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="F156" s="0" t="n">
+        <v>3.34</v>
+      </c>
+      <c r="G156" s="0" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="H156" s="0" t="n">
+        <v>9.68</v>
+      </c>
+      <c r="I156" s="0" t="n">
+        <v>7.14</v>
+      </c>
+      <c r="J156" s="0" t="n">
+        <v>8.609999999999999</v>
+      </c>
+      <c r="K156" s="0" t="n">
+        <v>5.36</v>
+      </c>
+      <c r="L156" s="0" t="n">
+        <v>8.19</v>
+      </c>
+      <c r="M156" s="0" t="n">
+        <v>3.38</v>
+      </c>
+      <c r="N156" s="0" t="n">
+        <v>9.35</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="1" t="n">
         <v>46158</v>
       </c>
+      <c r="B157" s="0" t="n">
+        <v>5.29</v>
+      </c>
+      <c r="C157" s="0" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="D157" s="0" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="E157" s="0" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="F157" s="0" t="n">
+        <v>1.94</v>
+      </c>
+      <c r="G157" s="0" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="H157" s="0" t="n">
+        <v>11.09</v>
+      </c>
+      <c r="I157" s="0" t="n">
+        <v>5.47</v>
+      </c>
+      <c r="J157" s="0" t="n">
+        <v>1.85</v>
+      </c>
+      <c r="K157" s="0" t="n">
+        <v>1.21</v>
+      </c>
+      <c r="L157" s="0" t="n">
+        <v>5.59</v>
+      </c>
+      <c r="M157" s="0" t="n">
+        <v>3.16</v>
+      </c>
+      <c r="N157" s="0" t="n">
+        <v>12.51</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="1" t="n">
         <v>46159</v>
       </c>
+      <c r="B158" s="0" t="n">
+        <v>7.95</v>
+      </c>
+      <c r="C158" s="0" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="D158" s="0" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="E158" s="0" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="F158" s="0" t="n">
+        <v>-0.14</v>
+      </c>
+      <c r="G158" s="0" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="H158" s="0" t="n">
+        <v>10.84</v>
+      </c>
+      <c r="I158" s="0" t="n">
+        <v>8.65</v>
+      </c>
+      <c r="J158" s="0" t="n">
+        <v>1.84</v>
+      </c>
+      <c r="K158" s="0" t="n">
+        <v>-0.36</v>
+      </c>
+      <c r="L158" s="0" t="n">
+        <v>1.21</v>
+      </c>
+      <c r="M158" s="0" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="N158" s="0" t="n">
+        <v>10.15</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="1" t="n">
         <v>46160</v>
+      </c>
+      <c r="B159" t="n">
+        <v>6.86</v>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="F159" t="n">
+        <v>1.82</v>
+      </c>
+      <c r="G159" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="H159" t="n">
+        <v>9.130000000000001</v>
+      </c>
+      <c r="I159" t="n">
+        <v>7.51</v>
+      </c>
+      <c r="J159" t="n">
+        <v>3.86</v>
+      </c>
+      <c r="K159" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="L159" t="n">
+        <v>2.21</v>
+      </c>
+      <c r="M159" t="n">
+        <v>2.06</v>
+      </c>
+      <c r="N159" t="n">
+        <v>8.699999999999999</v>
       </c>
     </row>
     <row r="160">

</xml_diff>